<commit_message>
feat: add track selection display toggle & remove banner text
</commit_message>
<xml_diff>
--- a/frontend/data/registrations.xlsx
+++ b/frontend/data/registrations.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Track Number</t>
   </si>
@@ -26,6 +26,18 @@
   </si>
   <si>
     <t>Leader Name</t>
+  </si>
+  <si>
+    <t>02</t>
+  </si>
+  <si>
+    <t>ver</t>
+  </si>
+  <si>
+    <t>Supply Chain Intelligence</t>
+  </si>
+  <si>
+    <t>verv</t>
   </si>
 </sst>
 </file>
@@ -71,10 +83,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -415,7 +430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -442,6 +457,23 @@
         <v>4</v>
       </c>
     </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>